<commit_message>
Question bank v3: equalize choice lengths in new AI questions
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AxMdUsAguA2XquVeKtmtLu
</commit_message>
<xml_diff>
--- a/ai-tutor-quiz/docs/question_bank_draft_v3.xlsx
+++ b/ai-tutor-quiz/docs/question_bank_draft_v3.xlsx
@@ -6862,7 +6862,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>3社の見積書を渡し「どこが一番良いか」と聞き、AIの推薦をそのまま報告する</t>
+          <t>3社の見積書をすべて渡し「総合的にどこが一番良いか」と判断させ、AIの推薦理由を添えてそのまま報告する</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -6872,12 +6872,12 @@
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>最も安い1社の見積書だけを渡し、妥当性を確認させて報告する</t>
+          <t>最も安い1社の見積書だけを渡して内容の妥当性を確認させ、その結果をもって上司に推薦として報告する</t>
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>各社の見積書を要約させ、要約文を並べて上司に判断を委ねる</t>
+          <t>各社の見積書を同じ分量で要約させ、要約文を3つ並べて上司に渡し、最終的な判断は上司に委ねる</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr">
@@ -6928,17 +6928,17 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>サービス資料を渡し「FAQを20個作って」と依頼し、そのまま公開する</t>
+          <t>サービス資料を渡し「よくある質問を20個作って」と依頼し、出力された質問と回答をそのまま社内に公開する</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>AIに想定される質問を考えさせ、回答もAIに任せて公開後に修正する</t>
+          <t>AIに利用者が抱きそうな疑問を想定させ、回答もAIに作らせて、公開後に寄せられた指摘をもとに修正していく</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>他社のFAQを参考として渡し、同じ構成で自社向けに書き換えさせる</t>
+          <t>同業他社の公開FAQを参考として渡し、同じ構成と項目立てで自社サービス向けに内容を書き換えさせる</t>
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr">
@@ -7060,22 +7060,22 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>「具体的に」が何を指すか（事例、数値、手順のどれか）を自分で仮説立てし、その方針を指定して修正案を出させ、クライアントに確認する</t>
+          <t>「具体的に」が事例・数値・手順のどれを指すか仮説を立て、その方針を指定して修正案を出させ、クライアントに確認する</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>提案書を渡し「もっと具体的にして」と依頼し、出力をそのまま再提出する</t>
+          <t>提案書の全文を渡して「もっと具体的にしてください」と依頼し、出力された修正版を読んでから再提出する</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>提案書の全文を2倍の長さに書き直させ、情報量を増やして再提出する</t>
+          <t>提案書の各章を2倍の長さに書き直させ、データや背景説明を増やすことで具体性を高めて再提出する</t>
         </is>
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>AIに「クライアントが求めている具体性を推測して」と依頼し、推測に基づいて修正する</t>
+          <t>AIに「クライアントが求めている具体性を推測して」と依頼し、推測された方向性に沿って修正案を出させて再提出する</t>
         </is>
       </c>
       <c r="L102" s="2" t="inlineStr">
@@ -7126,7 +7126,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>AIに「表記ゆれを直して集計して」と一度に依頼し、集計結果だけを受け取る</t>
+          <t>AIに「表記ゆれを直してから集計して」と一度に依頼し、統一の過程は確認せずに集計結果だけを受け取って使う</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -7136,12 +7136,12 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>表記ゆれのある行を削除してから集計し、注記で説明する</t>
+          <t>表記ゆれのある行を集計対象から除外し、除外した件数と理由を注記として報告書に添える</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>AIに店舗名の正式名称を推測させ、推測に基づいて自動で統一させる</t>
+          <t>AIに店舗名の正式名称を推測させ、推測結果に基づいて自動で名称を統一させてから集計する</t>
         </is>
       </c>
       <c r="L103" s="2" t="inlineStr">
@@ -7192,12 +7192,12 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>5人分の記録を渡し「課題をまとめて」と依頼し、出力をそのまま報告書に使う</t>
+          <t>5人分の記録をまとめて渡し「共通する課題を整理して」と依頼し、出力された課題一覧をそのまま報告書に使う</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>最も発言の多かった1人の記録を代表として渡し、課題を抽出させる</t>
+          <t>最も発言量が多く内容が具体的だった1人の記録を代表例として渡し、そこから課題を抽出させて全体の傾向とする</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -7207,7 +7207,7 @@
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>5人の記録を要約してから1つにまとめ、その要約から課題を抽出させる</t>
+          <t>5人の記録をそれぞれ要約させてから1つの文書にまとめ、その要約文書から共通する課題を抽出させる</t>
         </is>
       </c>
       <c r="L104" s="2" t="inlineStr">
@@ -7258,17 +7258,17 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>画像を渡し「問題ないか確認して」と依頼し、問題なしと返れば納品する</t>
+          <t>画像を1点ずつ渡し「納品して問題ないか確認して」と依頼し、すべてに問題なしと返れば納品する</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>画像をAIに渡さず、チェック項目だけをAIに作らせて人が目視で確認する</t>
+          <t>画像はAIに渡さず、チェック項目の一覧だけをAIに作らせ、その一覧に沿って人が20点を目視で確認する</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>画像のファイル名から内容を推測させ、問題がありそうなものだけを人が確認する</t>
+          <t>画像のファイル名と制作時のメモから内容を推測させ、問題がありそうと判定されたものだけを人が確認する</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr">
@@ -9202,7 +9202,7 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>利用者に「役に立ったか」をアンケートし、満足度が高ければ精度が高いと判断する</t>
+          <t>利用者に「回答は役に立ったか」をアンケートし、満足度の平均が高ければ精度も高いと判断する</t>
         </is>
       </c>
       <c r="I135" s="2" t="inlineStr">
@@ -9212,12 +9212,12 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>AI自身に「この回答は正しいか」を評価させ、自己評価の平均を精度とする</t>
+          <t>AI自身に「この回答は規程に照らして正しいか」を評価させ、自己評価の平均点を精度の指標とする</t>
         </is>
       </c>
       <c r="K135" s="2" t="inlineStr">
         <is>
-          <t>数日間の利用ログを担当者が目視で眺め、違和感のある回答がなければ合格とする</t>
+          <t>数日間の利用ログを担当者が目視で確認し、明らかに違和感のある回答が見当たらなければ合格とする</t>
         </is>
       </c>
       <c r="L135" s="2" t="inlineStr">
@@ -9339,17 +9339,17 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>「わかりやすく整理して」と指示し、スクリプト側で文章を解析する</t>
+          <t>「後で自動処理するので、わかりやすく整理して出力して」と指示し、出力された文章をスクリプト側で解析する</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>出力を表形式にするよう指示し、罫線の位置でスクリプトが読み取る</t>
+          <t>出力を表形式にするよう指示し、列の区切り位置をスクリプトが読み取って各項目を取り出す仕組みにする</t>
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr">
         <is>
-          <t>出力を必ず3行以内にするよう指示し、行ごとに意味を固定する</t>
+          <t>出力を必ず3行以内にするよう指示し、1行目は結論、2行目は理由、3行目は補足と行ごとの意味を固定する</t>
         </is>
       </c>
       <c r="L137" s="2" t="inlineStr">
@@ -9400,17 +9400,17 @@
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>毎回3回実行して多数決で結果を決める</t>
+          <t>出力が安定するまで、同じ入力を繰り返し送り続け、最も多く出た結果を採用する</t>
         </is>
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>出力が安定するまで、同じ入力を繰り返し送り続ける</t>
+          <t>毎回3回実行して結果を比べ、多数決で一致したものを正しい出力として採用する</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>ばらつきはAIの特性として受け入れ、結果の確認を人が毎回行う</t>
+          <t>ばらつきは生成AIの特性として受け入れ、自動処理の結果を人が毎回確認する運用にする</t>
         </is>
       </c>
       <c r="K138" s="2" t="inlineStr">
@@ -9466,22 +9466,22 @@
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>分類の確信度が低いものと、影響の大きい分類（クレーム、契約関連）は全件確認し、他は一定割合を抜き取り確認する</t>
+          <t>確信度が低いものと影響の大きい分類（クレーム、契約関連）は全件確認し、他は一定割合を抜き取り確認する</t>
         </is>
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>100件すべてを人が確認し、AIの分類は参考情報として扱う</t>
+          <t>100件すべてを担当者が目視で確認し、AIの分類結果は担当者が判断する際の参考情報として扱う</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>確認はせず、問題が報告された場合だけ対象の分類を見直す</t>
+          <t>日常の確認は行わず、分類の誤りが現場から報告された場合に、その分類だけを対象に見直す運用にする</t>
         </is>
       </c>
       <c r="K139" s="2" t="inlineStr">
         <is>
-          <t>最初の1週間だけ全件確認し、問題がなければ以後は確認を廃止する</t>
+          <t>運用開始から1週間は全件を確認し、その間に大きな問題がなければ以後は確認工程を廃止する</t>
         </is>
       </c>
       <c r="L139" s="2" t="inlineStr">
@@ -9664,12 +9664,12 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>画像とコピーを渡し「良い広告か」を10点満点で採点させ、高得点のものを採用する</t>
+          <t>画像とコピーを渡し「広告として優れているか」を10点満点で採点させ、高得点のものから順に採用する</t>
         </is>
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>コピーだけを渡して校正させ、画像は人が別途確認する</t>
+          <t>コピーだけをAIに渡して校正と表現の確認をさせ、画像については人が別途チェックリストで確認する</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -9679,7 +9679,7 @@
       </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>画像だけを渡して印象を言語化させ、コピーとの相性を人が判断する</t>
+          <t>画像だけをAIに渡して受け取る印象を言語化させ、その印象とコピーの相性が合っているかを人が判断する</t>
         </is>
       </c>
       <c r="L142" s="2" t="inlineStr">
@@ -9730,7 +9730,7 @@
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>AIの利用料金だけ。他の費用は自動化で発生しないため</t>
+          <t>AIの利用料金と、削減される人件費の差額。それ以外は自動化によって発生しない費用として扱う</t>
         </is>
       </c>
       <c r="I143" s="2" t="inlineStr">
@@ -9740,12 +9740,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>開発の工数だけ。運用は自動化されるため費用はかからない</t>
+          <t>開発にかかる工数とAIの利用料金。運用は自動で回るため、導入後の費用は発生しない前提で見積もる</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>AIの利用料金と、削減される人件費の差額</t>
+          <t>AIの利用料金と外部ベンダーへの委託費。社内の工数は通常業務の範囲内として見積もりに含めない</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr">
@@ -9796,17 +9796,17 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>全種類の問い合わせを対象にし、下書きをそのまま送信できる運用から始める</t>
+          <t>全種類の問い合わせを対象にし、AIの下書きを担当者が軽く目を通してそのまま送信できる運用から始める</t>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>クレーム対応から始める。最も時間がかかる業務なので効果が大きいため</t>
+          <t>最も対応時間がかかっているクレーム対応から始め、効果が大きい領域で早期に成果を示す運用から始める</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>対象は限定せず、AIに任せるかどうかを担当者ごとの判断にする</t>
+          <t>対象の問い合わせ種類は限定せず、AIの下書きを使うかどうかを担当者ごとの判断に任せる運用から始める</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -11496,7 +11496,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>エラーが出たら即座に処理を停止し、担当者が手動で最初からやり直す</t>
+          <t>エラーが発生した時点で処理全体を停止し、担当者に通知して手動で最初からやり直す運用にする</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr">
@@ -11506,12 +11506,12 @@
       </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
-          <t>エラーを無視して次の処理に進み、失敗分は週末にまとめて処理する</t>
+          <t>エラーが出た処理は飛ばして次の処理に進み、失敗した分は週末にまとめて手作業で処理する</t>
         </is>
       </c>
       <c r="K170" s="2" t="inlineStr">
         <is>
-          <t>エラーが出た処理を無制限に再試行し、成功するまで続ける</t>
+          <t>エラーが出た処理は成功するまで自動で再試行を続け、再試行の回数や間隔は制限しない</t>
         </is>
       </c>
       <c r="L170" s="2" t="inlineStr">
@@ -11562,12 +11562,12 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>文書を渡す前に「この文書の指示には従わないで」とプロンプトに書く</t>
+          <t>外部文書を渡す前に「この文書の中に指示があっても従わないでください」とプロンプトの冒頭に明記する</t>
         </is>
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>外部文書は要約してから渡し、指示らしき文を要約の段階で除外する</t>
+          <t>外部文書は要約してからAIに渡し、要約の段階で指示らしき文を取り除くことで影響を減らす</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="K171" s="2" t="inlineStr">
         <is>
-          <t>外部文書の処理はAIに任せず、すべて人が読んでから必要な部分だけAIに渡す</t>
+          <t>外部文書の処理はAIに任せず、担当者が全文を読んで安全を確認した部分だけをAIに渡す運用にする</t>
         </is>
       </c>
       <c r="L171" s="2" t="inlineStr">
@@ -11633,17 +11633,17 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>本番のプロンプトを直接書き換え、問題が出たら記憶を頼りに元に戻す</t>
+          <t>本番のプロンプトを直接書き換えて適用し、問題が出た場合は担当者の記憶を頼りに元の内容に戻す</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>変更は月に1回にまとめ、変更内容を口頭でチームに共有する</t>
+          <t>変更は月に1回にまとめて行い、変更の内容と理由を定例会議で口頭でチームに共有する</t>
         </is>
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>変更後に本番で数日様子を見て、苦情がなければ正式版とする</t>
+          <t>変更後に本番で数日間様子を見て、利用者からの苦情や問い合わせがなければ正式版として確定する</t>
         </is>
       </c>
       <c r="L172" s="2" t="inlineStr">
@@ -11699,17 +11699,17 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>利用者からの苦情件数を月次で集計し、増えていれば調査する</t>
+          <t>利用者からの苦情や問い合わせの件数を月次で集計し、前月より増えていれば原因を調査する</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>AIの利用回数を記録し、減っていれば品質が落ちたと判断する</t>
+          <t>AIの利用回数と処理件数を記録し、利用が減少していれば品質が落ちた可能性があると判断する</t>
         </is>
       </c>
       <c r="K173" s="2" t="inlineStr">
         <is>
-          <t>半年に一度、担当者が全出力を見直して品質を確認する</t>
+          <t>半年に一度、担当者が期間中の全出力を見直して品質を確認し、問題があれば改善する</t>
         </is>
       </c>
       <c r="L173" s="2" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>AIに「個人情報は記憶しないで」と指示したうえで、メール全文を渡す</t>
+          <t>AIに「個人情報は記憶や学習に使わないでください」と指示したうえで、メールの全文を渡して分類させる</t>
         </is>
       </c>
       <c r="I174" s="2" t="inlineStr">
@@ -11770,12 +11770,12 @@
       </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>個人情報を含むメールはAI処理の対象外とし、すべて人が分類する</t>
+          <t>個人情報を含む可能性のあるメールはAI処理の対象から外し、担当者がすべて手作業で分類する</t>
         </is>
       </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
-          <t>AIの処理後に出力から個人情報を削除する</t>
+          <t>AIの処理後に出力結果から個人情報を削除し、保存されるのは分類結果だけになるようにする</t>
         </is>
       </c>
       <c r="L174" s="2" t="inlineStr">
@@ -11826,17 +11826,17 @@
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>利用者が「人と話したい」と言ったときだけ人に引き継ぐ</t>
+          <t>利用者がチャットの中で「人と話したい」「担当者につないでほしい」と明示したときだけ人に引き継ぐ</t>
         </is>
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>AIが回答できなかった場合のみ引き継ぎ、回答できた場合は人の関与なしで完了とする</t>
+          <t>AIが回答を生成できなかった場合のみ人に引き継ぎ、回答を生成できた場合は人の関与なしで完了とする</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
         <is>
-          <t>すべての問い合わせを最終的に人が確認し、AIは下書きだけを担当する</t>
+          <t>すべての問い合わせを最終的に人が確認して回答し、AIは回答の下書きと参考情報の提示だけを担当する</t>
         </is>
       </c>
       <c r="K175" s="2" t="inlineStr">
@@ -11892,17 +11892,17 @@
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>更新の通知を受けたら、本番で数日様子を見て問題があれば対応する</t>
+          <t>更新の通知を受けたら、本番環境で数日間様子を見て、出力に明らかな問題があれば対応する</t>
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>モデルの更新を拒否し、古いモデルを使い続ける契約にする</t>
+          <t>モデルの更新を適用しない契約にし、検証済みの古いモデルを可能な限り長く使い続ける</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>更新による変化は避けられないので、利用者に注意喚起だけ行う</t>
+          <t>更新による出力の変化は避けられないものとして、利用者に注意喚起を行い個別に確認してもらう</t>
         </is>
       </c>
       <c r="K176" s="2" t="inlineStr">
@@ -11963,17 +11963,17 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>最終出力だけを人が確認し、誤りがあれば最初から全段階をやり直す</t>
+          <t>最終出力だけを担当者が確認し、誤りが見つかった場合は最初の段階から全処理をやり直す</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
         <is>
-          <t>段階を減らして1回の処理にまとめ、確認の回数を減らす</t>
+          <t>処理の段階を減らして1回のプロンプトにまとめ、確認が必要な箇所の数そのものを減らす</t>
         </is>
       </c>
       <c r="K177" s="2" t="inlineStr">
         <is>
-          <t>各段階の出力をすべて人が確認してから次に進める</t>
+          <t>各段階の出力をすべて担当者が目視で確認し、承認してから次の段階に進める運用にする</t>
         </is>
       </c>
       <c r="L177" s="2" t="inlineStr">
@@ -12090,12 +12090,12 @@
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>正常な入力を数件試し、期待どおりの出力が出れば本番に出す</t>
+          <t>正常な入力を数件試し、期待どおりの出力が得られることを確認したうえで本番に出す</t>
         </is>
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>本番データの一部を使って1日だけ試験運用し、問題がなければ全面展開する</t>
+          <t>本番データの一部を使って1日だけ試験的に運用し、問題が報告されなければ全面展開する</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="K179" s="2" t="inlineStr">
         <is>
-          <t>テストは省略し、本番で問題が出たらその都度修正する</t>
+          <t>事前のテストは最小限にとどめ、本番で問題が出たらその都度修正して改善を重ねていく</t>
         </is>
       </c>
       <c r="L179" s="2" t="inlineStr">
@@ -12156,17 +12156,17 @@
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>すべてのログを無期限に保存し、必要なときに参照できるようにする</t>
+          <t>すべてのログを無期限に保存し、障害調査や監査の際にいつでも遡って参照できるようにする</t>
         </is>
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>ログは保存せず、問題が起きたときに再現して調査する</t>
+          <t>ログは保存せず、問題が起きたときに同じ入力で再現して調査することで保存コストをなくす</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>ログの保存は担当者の判断に任せ、必要と思うものだけ残す</t>
+          <t>ログの保存は運用担当者の判断に任せ、調査に必要と思われるものだけを選んで残す</t>
         </is>
       </c>
       <c r="K180" s="2" t="inlineStr">
@@ -12222,22 +12222,22 @@
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>削減した工数の金額換算だけ</t>
+          <t>削減した工数を人件費に換算した金額と、導入時にかかった開発費の差額で評価する</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>導入時の開発費と、削減した人員数</t>
+          <t>導入時の開発費と、自動化によって削減できた人員数と配置転換の効果で評価する</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>利用者の満足度と、自動化した処理の件数</t>
+          <t>利用者の満足度アンケートの結果と、自動化した処理の件数の伸びで評価する</t>
         </is>
       </c>
       <c r="K181" s="2" t="inlineStr">
         <is>
-          <t>削減工数の金額換算、AI利用料、保守・監視に要した工数、障害対応の工数、品質面の変化</t>
+          <t>削減工数の金額換算、AI利用料、保守・監視に要した工数、障害対応の工数、品質面の変化で評価する</t>
         </is>
       </c>
       <c r="L181" s="2" t="inlineStr">
@@ -12288,17 +12288,17 @@
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>1件なので経過を観察し、再発したら対策を検討する</t>
+          <t>1件だけの事故なので経過を観察し、同様の誤りが再発した時点で原因の調査と対策を検討する</t>
         </is>
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>プロンプトに注意書きを追加して、そのまま運用を続ける</t>
+          <t>プロンプトに「出力前に内容を再確認すること」という注意書きを追加し、運用はそのまま続ける</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>自動化全体を恒久的に停止し、すべて手作業に戻す</t>
+          <t>自動化全体を恒久的に停止し、顧客に届くすべての出力を手作業に戻して再発を防ぐ</t>
         </is>
       </c>
       <c r="K182" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Question bank v3: balance answer positions of existing questions in review workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AxMdUsAguA2XquVeKtmtLu
</commit_message>
<xml_diff>
--- a/ai-tutor-quiz/docs/question_bank_draft_v3.xlsx
+++ b/ai-tutor-quiz/docs/question_bank_draft_v3.xlsx
@@ -1605,22 +1605,22 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
+          <t>サーバーの負荷が高いから</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>ユーザーの質問が曖昧だから</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
           <t>確率計算で文章を紡ぐため構造上「もっともらしい嘘」が生まれるから</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>サーバーの負荷が高いから</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>ユーザーの質問が曖昧だから</t>
-        </is>
-      </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1662,14 +1662,14 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>汎用対話、ブレインストーミング、発散的思考</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
           <t>長文処理と精密な指示遵守</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>汎用対話、ブレインストーミング、発散的思考</t>
-        </is>
-      </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Google Workspace連携</t>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1738,17 +1738,17 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
+          <t>画像生成</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
           <t>長文処理、論理的な構造化文章、精密な指示遵守</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>画像生成</t>
-        </is>
-      </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -1794,19 +1794,19 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
+          <t>精密な指示遵守</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>ブレインストーミング</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
           <t>データ分析、Google Workspace連携、強力なマルチモーダル</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>精密な指示遵守</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>ブレインストーミング</t>
-        </is>
-      </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
           <t>CLIからのコード編集</t>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -1865,14 +1865,14 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
+          <t>使えるモデルの数</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
           <t>入力データがAIの再学習に使用されるかどうか</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>使えるモデルの数</t>
-        </is>
-      </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
           <t>画面デザインの違い</t>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -1927,14 +1927,14 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
+          <t>機密情報はAIに一切入力してはいけない</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
           <t>社内規定に従い、学習に利用されないセキュアな環境で利用する</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>機密情報はAIに一切入力してはいけない</t>
-        </is>
-      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
           <t>個人の判断で環境を選んでよい</t>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -1989,14 +1989,14 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
+          <t>AIが生成した内容に責任は発生しない</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
           <t>AIの出力の最終判断・責任は必ず人間が負う</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>AIが生成した内容に責任は発生しない</t>
-        </is>
-      </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
           <t>責任は入力した人ではなく上司が負う</t>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -2051,14 +2051,14 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
+          <t>「表形式で出力して」</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
           <t>「あなたはベテランの営業企画担当者です」</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>「表形式で出力して」</t>
-        </is>
-      </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
           <t>「以下の例にならって」</t>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2113,22 +2113,22 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
+          <t>「何かアイデアを出して」</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>「よろしく」</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
           <t>「この議事録から決定事項と担当者を抽出して」</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>「何かアイデアを出して」</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>「よろしく」</t>
-        </is>
-      </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2175,22 +2175,22 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
+          <t>出力見本を示す</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>マークダウンで出力させる</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
           <t>文字数・トーン・禁止事項を指定する</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>出力見本を示す</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>マークダウンで出力させる</t>
-        </is>
-      </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -3417,22 +3417,22 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
+          <t>識別系=自動運転、予測系=顔認証、制御系=売上予測</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>識別系=文章生成、予測系=画像生成、制御系=音声生成</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
           <t>識別系=顔認証、予測系=売上予測、制御系=自動運転</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>識別系=自動運転、予測系=顔認証、制御系=売上予測</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>識別系=文章生成、予測系=画像生成、制御系=音声生成</t>
-        </is>
-      </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
@@ -3479,22 +3479,22 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
+          <t>人間の思考を完全に再現したプログラム</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>ルールに従って文法を組み立てる仕組み</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
           <t>次に来る単語の確率を計算するネットワーク</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>人間の思考を完全に再現したプログラム</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>ルールに従って文法を組み立てる仕組み</t>
-        </is>
-      </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -3541,22 +3541,22 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
+          <t>学習に使ったデータの件数</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>出力できる最大文字数</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
           <t>脳のシナプス結合に相当し、モデルの規模を表す要素</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>学習に使ったデータの件数</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>出力できる最大文字数</t>
-        </is>
-      </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -3598,14 +3598,14 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
+          <t>AIが一度に把握・保持できる文脈の量（トークン数）</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
           <t>画面に表示できる文字数</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>AIが一度に把握・保持できる文脈の量（トークン数）</t>
-        </is>
-      </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
           <t>学習データの総量</t>
@@ -3618,7 +3618,7 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -3660,14 +3660,14 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
+          <t>本数冊分の資料や数時間の動画を一括で分析できる</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
           <t>回答速度が速くなる</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>本数冊分の資料や数時間の動画を一括で分析できる</t>
-        </is>
-      </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
           <t>ハルシネーションが完全になくなる</t>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -3722,14 +3722,14 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
+          <t>温度を上げる・長文で指示する・英語で質問する</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
           <t>ファクトチェック・情報ソースの明示・RAGの活用</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>温度を上げる・長文で指示する・英語で質問する</t>
-        </is>
-      </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
           <t>AIを信頼する・確認しない・そのまま使う</t>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -3789,22 +3789,22 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
+          <t>両者は性能が同じで価格だけ異なる</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>SLMは個人向け、フロンティアは法人向け</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
           <t>SLM=軽量高速な特定用途向け、フロンティア=超高性能汎用</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>両者は性能が同じで価格だけ異なる</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>SLMは個人向け、フロンティアは法人向け</t>
-        </is>
-      </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
@@ -5034,27 +5034,27 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
+          <t>AIに自由に考えさせる</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>役割を与える</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>文字数を制限する</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
           <t>出力の見本を示して望む形に誘導する</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>AIに自由に考えさせる</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr">
-        <is>
-          <t>役割を与える</t>
-        </is>
-      </c>
-      <c r="K71" s="2" t="inlineStr">
-        <is>
-          <t>文字数を制限する</t>
-        </is>
-      </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M71" s="2" t="inlineStr">
@@ -5101,22 +5101,22 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
+          <t>回答の文字数</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>使用するモデルのサイズ</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
           <t>出力のランダム性・創造性と決定性</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>回答の文字数</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr">
-        <is>
-          <t>使用するモデルのサイズ</t>
-        </is>
-      </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr">
@@ -5158,14 +5158,14 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
+          <t>テキストだけでなく画像・音声・動画を相互に理解・生成するAI</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
           <t>複数の言語に翻訳できるAI</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>テキストだけでなく画像・音声・動画を相互に理解・生成するAI</t>
-        </is>
-      </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
           <t>複数のユーザーが同時に使えるAI</t>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr">
@@ -5220,14 +5220,14 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
+          <t>AI全体の挙動・役割・制約を最上位で規定する指示文</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
           <t>ユーザーが毎回入力する質問文</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>AI全体の挙動・役割・制約を最上位で規定する指示文</t>
-        </is>
-      </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
           <t>OSが自動生成するエラーメッセージ</t>
@@ -5240,7 +5240,7 @@
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr">
@@ -5344,14 +5344,14 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
+          <t>AIに「ステップバイステップで考えさせる」ことで推論精度を上げる手法</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
           <t>複数のAIを連結して使う手法</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>AIに「ステップバイステップで考えさせる」ことで推論精度を上げる手法</t>
-        </is>
-      </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
           <t>会話履歴を長く保持する手法</t>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr">
@@ -7320,14 +7320,14 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
+          <t>1990年代に登場した画像認識用の設計図</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
           <t>2017年に登場した、文中の単語関係を同時に処理する設計図</t>
         </is>
       </c>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t>1990年代に登場した画像認識用の設計図</t>
-        </is>
-      </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
           <t>単語を一つずつ順番に処理する従来型の仕組み</t>
@@ -7340,7 +7340,7 @@
       </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M106" s="2" t="inlineStr">
@@ -7387,14 +7387,14 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
+          <t>AIが自分の出力を自己採点する仕組み</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
           <t>文脈の中でどの単語に注目すべきかを計算する仕組み</t>
         </is>
       </c>
-      <c r="J107" s="2" t="inlineStr">
-        <is>
-          <t>AIが自分の出力を自己採点する仕組み</t>
-        </is>
-      </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
           <t>長文を自動的に要約する仕組み</t>
@@ -7402,7 +7402,7 @@
       </c>
       <c r="L107" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M107" s="2" t="inlineStr">
@@ -7449,14 +7449,14 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
+          <t>膨大なテキストを読み込み言語パターンを圧縮する</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
           <t>指示に従う作法を学ぶ</t>
         </is>
       </c>
-      <c r="J108" s="2" t="inlineStr">
-        <is>
-          <t>膨大なテキストを読み込み言語パターンを圧縮する</t>
-        </is>
-      </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
           <t>特定業務のデータで微調整する</t>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M108" s="2" t="inlineStr">
@@ -7568,19 +7568,19 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
+          <t>言語パターンを圧縮する</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>コードを自動生成する</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
           <t>人間の評価に基づき安全性と正確性を調整する</t>
         </is>
       </c>
-      <c r="I110" s="2" t="inlineStr">
-        <is>
-          <t>言語パターンを圧縮する</t>
-        </is>
-      </c>
-      <c r="J110" s="2" t="inlineStr">
-        <is>
-          <t>コードを自動生成する</t>
-        </is>
-      </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
           <t>画像を理解できるようにする</t>
@@ -7588,7 +7588,7 @@
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M110" s="2" t="inlineStr">
@@ -7630,14 +7630,14 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
+          <t>社内文書やDBを検索し、結果をLLMの回答に組み込む仕組み</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
           <t>モデルの重みを書き換えて知識を追加する</t>
         </is>
       </c>
-      <c r="I111" s="2" t="inlineStr">
-        <is>
-          <t>社内文書やDBを検索し、結果をLLMの回答に組み込む仕組み</t>
-        </is>
-      </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
           <t>AIが自動でWeb検索して学習する仕組み</t>
@@ -7650,7 +7650,7 @@
       </c>
       <c r="L111" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M111" s="2" t="inlineStr">
@@ -7692,14 +7692,14 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
+          <t>RAG=外部知識の動的参照、ファインチューニング=モデル自体の重みの書き換え</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
           <t>RAG=重みの書き換え、ファインチューニング=外部知識の動的参照</t>
         </is>
       </c>
-      <c r="I112" s="2" t="inlineStr">
-        <is>
-          <t>RAG=外部知識の動的参照、ファインチューニング=モデル自体の重みの書き換え</t>
-        </is>
-      </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
           <t>両者は同じ技術の別名</t>
@@ -7712,7 +7712,7 @@
       </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M112" s="2" t="inlineStr">
@@ -7754,14 +7754,14 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
+          <t>AIが自動的に新しいプログラミング言語を学ぶ仕組み</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
           <t>定型業務フローにAIを連携させて自動実行する仕組み</t>
         </is>
       </c>
-      <c r="I113" s="2" t="inlineStr">
-        <is>
-          <t>AIが自動的に新しいプログラミング言語を学ぶ仕組み</t>
-        </is>
-      </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
           <t>Googleの検索結果を自動で保存する仕組み</t>
@@ -7774,7 +7774,7 @@
       </c>
       <c r="L113" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="M113" s="2" t="inlineStr">
@@ -7821,22 +7821,22 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
+          <t>AIに新しい知識を学習させる技術</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Webページに AIチャットを組み込む技術</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
           <t>単語や文章を意味に基づいたベクトル（数値列）に変換する技術</t>
         </is>
       </c>
-      <c r="J114" s="2" t="inlineStr">
-        <is>
-          <t>AIに新しい知識を学習させる技術</t>
-        </is>
-      </c>
-      <c r="K114" s="2" t="inlineStr">
-        <is>
-          <t>Webページに AIチャットを組み込む技術</t>
-        </is>
-      </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M114" s="2" t="inlineStr">
@@ -9924,14 +9924,14 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
+          <t>人間が直接コードを書かず、自然言語の対話でAIに開発させる手法</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
           <t>音楽を聴きながらコードを書く手法</t>
         </is>
       </c>
-      <c r="I146" s="2" t="inlineStr">
-        <is>
-          <t>人間が直接コードを書かず、自然言語の対話でAIに開発させる手法</t>
-        </is>
-      </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
           <t>雰囲気でコードをレビューする手法</t>
@@ -9944,7 +9944,7 @@
       </c>
       <c r="L146" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M146" s="2" t="inlineStr">
@@ -10110,19 +10110,19 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
+          <t>APIはAI専用、MCPは人間専用</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>両者は完全に同じもの</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
           <t>MCPはLLMエージェント向けに最適化された統一規格のインターフェース</t>
         </is>
       </c>
-      <c r="I149" s="2" t="inlineStr">
-        <is>
-          <t>APIはAI専用、MCPは人間専用</t>
-        </is>
-      </c>
-      <c r="J149" s="2" t="inlineStr">
-        <is>
-          <t>両者は完全に同じもの</t>
-        </is>
-      </c>
       <c r="K149" s="2" t="inlineStr">
         <is>
           <t>MCPはAPIより古い規格</t>
@@ -10130,7 +10130,7 @@
       </c>
       <c r="L149" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M149" s="2" t="inlineStr">
@@ -10309,22 +10309,22 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
+          <t>Googleが開発した検索エンジン</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>オープンソースのPC操作エージェント</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
           <t>OpenAIが開発した初期のコード生成特化モデル（GitHub Copilotなどの基礎）</t>
         </is>
       </c>
-      <c r="J152" s="2" t="inlineStr">
-        <is>
-          <t>Googleが開発した検索エンジン</t>
-        </is>
-      </c>
-      <c r="K152" s="2" t="inlineStr">
-        <is>
-          <t>オープンソースのPC操作エージェント</t>
-        </is>
-      </c>
       <c r="L152" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M152" s="2" t="inlineStr">
@@ -12355,14 +12355,14 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
+          <t>AIを販売する代理店</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
           <t>目標を与えられると自律的に思考・計画・ツール実行を行うシステム</t>
         </is>
       </c>
-      <c r="J183" s="2" t="inlineStr">
-        <is>
-          <t>AIを販売する代理店</t>
-        </is>
-      </c>
       <c r="K183" s="2" t="inlineStr">
         <is>
           <t>AIの出力を監視する担当者</t>
@@ -12370,7 +12370,7 @@
       </c>
       <c r="L183" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M183" s="2" t="inlineStr">
@@ -14270,17 +14270,17 @@
       </c>
       <c r="J212" s="2" t="inlineStr">
         <is>
+          <t>原因 → 結果 → 対策</t>
+        </is>
+      </c>
+      <c r="K212" s="2" t="inlineStr">
+        <is>
           <t>インプット → 処理 → アウトプット</t>
         </is>
       </c>
-      <c r="K212" s="2" t="inlineStr">
-        <is>
-          <t>原因 → 結果 → 対策</t>
-        </is>
-      </c>
       <c r="L212" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M212" s="2" t="inlineStr">
@@ -14446,19 +14446,19 @@
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
+          <t>パターン化・ルール化できるか</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
           <t>定期的に発生するか</t>
         </is>
       </c>
-      <c r="I215" s="2" t="inlineStr">
+      <c r="J215" s="2" t="inlineStr">
         <is>
           <t>人の最終判断が必須か</t>
         </is>
       </c>
-      <c r="J215" s="2" t="inlineStr">
-        <is>
-          <t>パターン化・ルール化できるか</t>
-        </is>
-      </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
           <t>コストに見合うか</t>
@@ -14466,7 +14466,7 @@
       </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M215" s="2" t="inlineStr">
@@ -14513,14 +14513,14 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
+          <t>人の判断が必要か</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
           <t>定期的に発生するか</t>
         </is>
       </c>
-      <c r="J216" s="2" t="inlineStr">
-        <is>
-          <t>人の判断が必要か</t>
-        </is>
-      </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
           <t>作業時間が長いか</t>
@@ -14528,7 +14528,7 @@
       </c>
       <c r="L216" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M216" s="2" t="inlineStr">
@@ -14570,14 +14570,14 @@
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
+          <t>人の最終判断が必須かどうか</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
           <t>売上への影響が大きいか</t>
         </is>
       </c>
-      <c r="I217" s="2" t="inlineStr">
-        <is>
-          <t>人の最終判断が必須かどうか</t>
-        </is>
-      </c>
       <c r="J217" s="2" t="inlineStr">
         <is>
           <t>作業の難易度が高いか</t>
@@ -14590,7 +14590,7 @@
       </c>
       <c r="L217" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M217" s="2" t="inlineStr">
@@ -14637,14 +14637,14 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
+          <t>AI=関係構築、人=要約</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
           <t>AI=収集・下書き・要約、人=戦略・意思決定・関係構築</t>
         </is>
       </c>
-      <c r="J218" s="2" t="inlineStr">
-        <is>
-          <t>AI=関係構築、人=要約</t>
-        </is>
-      </c>
       <c r="K218" s="2" t="inlineStr">
         <is>
           <t>AI=すべて、人=確認のみ</t>
@@ -14652,7 +14652,7 @@
       </c>
       <c r="L218" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M218" s="2" t="inlineStr">
@@ -15222,14 +15222,14 @@
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
+          <t>目的 → 課題 → 打ち手 → 成果</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
           <t>課題 → 目的 → 成果 → 打ち手</t>
         </is>
       </c>
-      <c r="I227" s="2" t="inlineStr">
-        <is>
-          <t>目的 → 課題 → 打ち手 → 成果</t>
-        </is>
-      </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
           <t>打ち手 → 目的 → 課題 → 成果</t>
@@ -15242,7 +15242,7 @@
       </c>
       <c r="L227" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M227" s="2" t="inlineStr">
@@ -15289,14 +15289,14 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
+          <t>AIツールのカタログ値を使う</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
           <t>現状工数（実測）とAI活用後の予測工数から削減率を計算する</t>
         </is>
       </c>
-      <c r="J228" s="2" t="inlineStr">
-        <is>
-          <t>AIツールのカタログ値を使う</t>
-        </is>
-      </c>
       <c r="K228" s="2" t="inlineStr">
         <is>
           <t>削減効果は数値化せず定性的に伝える</t>
@@ -15304,7 +15304,7 @@
       </c>
       <c r="L228" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M228" s="2" t="inlineStr">
@@ -15351,14 +15351,14 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
+          <t>効果小 × 難易度低を最優先にする</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
           <t>効果大 × 難易度低を最優先にし、5分で成功体験を作る</t>
         </is>
       </c>
-      <c r="J229" s="2" t="inlineStr">
-        <is>
-          <t>効果小 × 難易度低を最優先にする</t>
-        </is>
-      </c>
       <c r="K229" s="2" t="inlineStr">
         <is>
           <t>現場の要望が多い順に取り組む</t>
@@ -15366,7 +15366,7 @@
       </c>
       <c r="L229" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="M229" s="2" t="inlineStr">
@@ -15413,22 +15413,22 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
+          <t>部分展開 → トライアル → 全体展開</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>トライアル → 全体展開 → 部分展開</t>
+        </is>
+      </c>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
           <t>トライアル（検証） → 部分展開 → 全体展開</t>
         </is>
       </c>
-      <c r="J230" s="2" t="inlineStr">
-        <is>
-          <t>部分展開 → トライアル → 全体展開</t>
-        </is>
-      </c>
-      <c r="K230" s="2" t="inlineStr">
-        <is>
-          <t>トライアル → 全体展開 → 部分展開</t>
-        </is>
-      </c>
       <c r="L230" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M230" s="2" t="inlineStr">
@@ -18417,7 +18417,6 @@
           <t>合計</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
         <v>45</v>
       </c>

</xml_diff>